<commit_message>
Deploy approved final Dinner menu update
</commit_message>
<xml_diff>
--- a/recipe-completeness-audit.xlsx
+++ b/recipe-completeness-audit.xlsx
@@ -84,8 +84,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompletenessAudit" displayName="CompletenessAudit" ref="A1:E7" totalsRowShown="0">
-  <autoFilter ref="A1:E7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompletenessAudit" displayName="CompletenessAudit" ref="A1:E5" totalsRowShown="0">
+  <autoFilter ref="A1:E5"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Recipe Name"/>
     <tableColumn id="2" name="Issue Type"/>
@@ -99,13 +99,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
-    <col min="4" max="4" width="55" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="55" customWidth="1"/>
   </cols>
   <sheetData>
@@ -139,12 +139,12 @@
     <row r="2" ht="45" customHeight="1">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">GAZPACHO SOUP</t>
+          <t xml:space="preserve">SUMMER MINESTRONE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ingredient quantity, name, or unit missing</t>
+          <t xml:space="preserve">Fewer than 3 ingredients</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="2">
@@ -154,7 +154,7 @@
       </c>
       <c r="D2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">https://artsincubator.ca/cookbook/recipes/soups/chilled-roasted-red-pepper-and-cucumber-gazpacho?gad_source=1&amp;gad_campaignid=23003435220&amp;gbraid=0AAAAA9TQSxmUYZLv5pmrvyhnvkhnj-kz4&amp;gclid=Cj0KCQjwof_QBhCgARIsADaMzOfTmj_KaDwXLP6VyuCBFY8dTZdVmUlZjjSQI-siB0nIOjIar33iRJ4aApEZEALw_wcB</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
@@ -166,12 +166,12 @@
     <row r="3" ht="45" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SOBA NOODLE SALAD</t>
+          <t xml:space="preserve">SUMMER MINESTRONE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ingredient quantity, name, or unit missing</t>
+          <t xml:space="preserve">Placeholder or generic ingredient</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="2">
@@ -181,7 +181,7 @@
       </c>
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">https://www.veganricha.com/cold-soba-noodle-salad-recipe/</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
@@ -198,7 +198,7 @@
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fewer than 3 ingredients</t>
+          <t xml:space="preserve">Fewer than 3 instructions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="2">
@@ -225,7 +225,7 @@
       </c>
       <c r="B5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Placeholder or generic ingredient</t>
+          <t xml:space="preserve">Placeholder or generic instruction</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="2">
@@ -244,62 +244,8 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">SUMMER MINESTRONE</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Fewer than 3 instructions</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Dinner recipe is shared with Lunch and was not modified due to the deployment restriction.</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual review required; Lunch record preserved unchanged.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">SUMMER MINESTRONE</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Placeholder or generic instruction</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Dinner recipe is shared with Lunch and was not modified due to the deployment restriction.</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual review required; Lunch record preserved unchanged.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:E5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>